<commit_message>
Cambios CSS, html, visualización en general.
</commit_message>
<xml_diff>
--- a/bateria_tests/estudios/plantilla_estudios_bueno_1solo.xlsx
+++ b/bateria_tests/estudios/plantilla_estudios_bueno_1solo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pablo\OneDrive\Documentos\Practicas_UOC\datos_muestras\bateria_tests\estudios\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2C73364-DB23-4916-B50F-73260C8C40F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C2DD638-1D48-45A4-B793-BA09C49D6A1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1060" yWindow="1060" windowWidth="20570" windowHeight="7450" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t>Descripción</t>
   </si>
@@ -49,6 +49,9 @@
   </si>
   <si>
     <t>desc</t>
+  </si>
+  <si>
+    <t>alfa</t>
   </si>
 </sst>
 </file>
@@ -100,10 +103,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -416,8 +420,8 @@
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A2">
-        <v>1</v>
+      <c r="A2" t="s">
+        <v>8</v>
       </c>
       <c r="B2">
         <v>1101012</v>
@@ -425,11 +429,11 @@
       <c r="C2" t="s">
         <v>7</v>
       </c>
-      <c r="D2">
-        <v>5</v>
-      </c>
-      <c r="E2">
-        <v>5</v>
+      <c r="D2" s="3">
+        <v>32964</v>
+      </c>
+      <c r="E2" s="3">
+        <v>36832</v>
       </c>
       <c r="F2" t="s">
         <v>6</v>

</xml_diff>